<commit_message>
feat: add Colab workflow and improve scheduling
</commit_message>
<xml_diff>
--- a/outputs/demo/easy_best_timetable.xlsx
+++ b/outputs/demo/easy_best_timetable.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>data/01_data_timetable.xlsx</t>
+          <t>data/instances/instance_easy.xlsx</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>01_data_timetable.xlsx</t>
+          <t>instance_easy.xlsx</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>data/01_data_timetable.xlsx</t>
+          <t>data/instances/instance_easy.xlsx</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>outputs/datasets/01_data_timetable.normalized.json</t>
+          <t>outputs/datasets/instance_easy.normalized.json</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>20.602957299910486</t>
+          <t>14.828526598999815</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>20.602957299910486</t>
+          <t>14.828526598999815</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 00:43:16</t>
+          <t>2026-09-01 16:29:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: remove Colab notebook and refresh demo outputs
</commit_message>
<xml_diff>
--- a/outputs/demo/easy_best_timetable.xlsx
+++ b/outputs/demo/easy_best_timetable.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>14.828526598999815</t>
+          <t>14.055336500000067</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>14.828526598999815</t>
+          <t>14.055336500000067</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 16:29:10</t>
+          <t>2026-09-03 15:07:37</t>
         </is>
       </c>
     </row>
@@ -24746,7 +24746,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -24813,7 +24813,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -24880,7 +24880,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -24947,7 +24947,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -25014,7 +25014,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -25081,7 +25081,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -25148,7 +25148,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -25215,7 +25215,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -25282,7 +25282,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -25349,7 +25349,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -25416,7 +25416,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -25483,7 +25483,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -25550,7 +25550,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -25617,7 +25617,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -25684,7 +25684,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -25751,7 +25751,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -25818,7 +25818,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -25885,7 +25885,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -25952,7 +25952,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -26019,7 +26019,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -26086,7 +26086,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -26153,7 +26153,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -26220,7 +26220,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -26287,7 +26287,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -26354,7 +26354,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -26421,7 +26421,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -26488,7 +26488,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -26555,7 +26555,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -26622,7 +26622,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -26689,7 +26689,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -26756,7 +26756,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -26823,7 +26823,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -26890,7 +26890,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -26957,7 +26957,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -27024,7 +27024,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -27091,7 +27091,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -27158,7 +27158,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -27225,7 +27225,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -27292,7 +27292,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -27359,7 +27359,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -27426,7 +27426,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -27493,7 +27493,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -27560,7 +27560,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -27627,7 +27627,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -27694,7 +27694,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -27761,7 +27761,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -27828,7 +27828,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -27895,7 +27895,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -27962,7 +27962,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -28029,7 +28029,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -28096,7 +28096,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -28163,7 +28163,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -28230,7 +28230,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -28297,7 +28297,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Giảm số ghế trống trong phòng</t>
+          <t>Giảm tỷ lệ ghế trống trong phòng</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -28842,7 +28842,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
-    <col width="859" customWidth="1" min="2" max="2"/>
+    <col width="850" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -28985,7 +28985,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>{"S1": {"enabled": true, "key": "compact_student_schedule", "name": "Giảm số ngày sinh viên phải đến trường", "weight": 10}, "S2": {"enabled": true, "key": "late_day_periods", "name": "Hạn chế quá nhiều tiết cuối ngày", "weight": 5}, "S3": {"enabled": true, "key": "preferred_shift_mismatch", "name": "Ưu tiên ca học mong muốn của lớp học phần", "weight": 4}, "S4": {"enabled": true, "key": "room_seat_waste", "name": "Giảm số ghế trống trong phòng", "weight": 2}, "S5": {"enabled": true, "key": "consecutive_cross_campus", "name": "Hạn chế giảng viên di chuyển liên tiếp giữa hai cơ sở", "weight": 8}, "S6": {"enabled": true, "key": "preferred_campus_mismatch", "name": "Ưu tiên cơ sở mong muốn của lớp học phần", "weight": 3}, "S7": {"enabled": true, "key": "student_home_campus_mismatch", "name": "Ưu tiên cơ sở chính của nhóm sinh viên", "weight": 4}}</t>
+          <t>{"S1": {"enabled": true, "key": "compact_student_schedule", "name": "Giảm số ngày sinh viên phải đến trường", "weight": 10}, "S2": {"enabled": true, "key": "late_day_periods", "name": "Hạn chế quá nhiều tiết cuối ngày", "weight": 5}, "S3": {"enabled": true, "key": "preferred_shift_mismatch", "name": "Ưu tiên ca học mong muốn của lớp học phần", "weight": 4}, "S4": {"enabled": true, "key": "room_seat_waste", "name": "Giảm tỷ lệ ghế trống trong phòng", "weight": 2}, "S5": {"enabled": true, "key": "consecutive_cross_campus", "name": "Hạn chế giảng viên chuyển cơ sở liên tiếp", "weight": 8}, "S6": {"enabled": true, "key": "preferred_campus_mismatch", "name": "Ưu tiên cơ sở mong muốn của lớp học phần", "weight": 3}, "S7": {"enabled": true, "key": "student_home_campus_mismatch", "name": "Ưu tiên cơ sở chính của nhóm sinh viên", "weight": 4}}</t>
         </is>
       </c>
     </row>

</xml_diff>